<commit_message>
Build q2342 Airflow Windows reproduction
</commit_message>
<xml_diff>
--- a/task/任务规格转化.xlsx
+++ b/task/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R249221f339854318"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="Rdbfdb02223114c1e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -333,7 +333,7 @@
         <x:v>原始输入文件</x:v>
       </x:c>
       <x:c r="B7" s="5" t="str">
-        <x:v>input_data/training_requests.csv、team_controls.csv、pool_plan.csv、rehearsal_scenarios.csv、release_policy.json、starter/shared_gpu_release_rehearsal_starter.py和数据说明.md</x:v>
+        <x:v>input_data/training_requests.csv、team_controls.csv、pool_plan.csv、rehearsal_scenarios.csv、release_policy.json、report_contract.csv、starter/shared_gpu_release_rehearsal_starter.py和数据说明.md</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -341,7 +341,7 @@
         <x:v>目标输出文件</x:v>
       </x:c>
       <x:c r="B8" s="5" t="str">
-        <x:v>dags和tools目录各一份Python文件，reports目录五份CSV，以及runtime_events目录中的场景事件</x:v>
+        <x:v>dags和tools目录各一份Python文件，reports目录五份CSV</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -349,7 +349,7 @@
         <x:v>核心操作链</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
-        <x:v>关联申请与团队控制→校验Pool及槽位→写入Airflow Pool→完成DAG结构→DagBag导入→运行两个场景→回读DagRun和TaskInstance→汇总租约事件</x:v>
+        <x:v>关联申请与团队控制→校验Pool及槽位→写入Airflow Pool→完成DAG结构→DagBag导入→运行两个场景→回读DagRun和TaskInstance→按报告合同汇总租约事件</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -357,7 +357,7 @@
         <x:v>输入一致性模块</x:v>
       </x:c>
       <x:c r="B10" s="5" t="str">
-        <x:v>业务主键唯一，团队和Pool外键存在，申请Pool符合团队权限，pool_slots不超过团队上限，失败对象属于申请集合</x:v>
+        <x:v>业务主键唯一，团队和Pool外键存在，申请Pool符合团队权限，pool_slots不超过团队上限，失败对象属于申请集合，报告合同路径与字段完整</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -381,7 +381,7 @@
         <x:v>任务资源模块</x:v>
       </x:c>
       <x:c r="B13" s="5" t="str">
-        <x:v>五个申请任务按release_order连接，pool和pool_slots逐行来自training_requests.csv</x:v>
+        <x:v>五个任务组标识逐行来自training_requests.csv，组内任务标识来自release_policy.json，申请任务按release_order连接，pool和pool_slots来自申请表</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
@@ -405,7 +405,7 @@
         <x:v>状态导出模块</x:v>
       </x:c>
       <x:c r="B16" s="5" t="str">
-        <x:v>从本次元数据库和DAG对象导出结构、Pool、场景、TaskInstance和事件报告，不用预期状态代替观测状态</x:v>
+        <x:v>按report_contract.csv从本次元数据库和DAG对象导出结构、Pool、场景、TaskInstance和事件报告，不用预期状态代替观测状态</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
@@ -413,7 +413,7 @@
         <x:v>完成条件</x:v>
       </x:c>
       <x:c r="B17" s="5" t="str">
-        <x:v>七项文件路径与runtime_events齐全，DAG可导入，两个场景状态符合输入，两个场景各释放一次租约，报告可反向连接本次Airflow对象</x:v>
+        <x:v>七项文件路径齐全且没有未列明目录，DAG可导入，两个场景状态符合输入，两个场景各释放一次租约，报告可反向连接本次Airflow对象</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">

</xml_diff>

<commit_message>
Replace authoring language with business source
</commit_message>
<xml_diff>
--- a/task/任务规格转化.xlsx
+++ b/task/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R126576f33f214eca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R1d0823ab937c44c4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -317,7 +317,7 @@
         <x:v>输入来源</x:v>
       </x:c>
       <x:c r="B5" s="5" t="str">
-        <x:v>训练平台发布值班提供的自造演练材料</x:v>
+        <x:v>训练平台发布值班提供的共享GPU窗口申请、资源池方案和发布策略</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">

</xml_diff>